<commit_message>
[EXIT] 2026-03-03 11:59 UTC
</commit_message>
<xml_diff>
--- a/trade_tracker.xlsx
+++ b/trade_tracker.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="₹#,##0;-₹#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0%;-0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +53,14 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,6 +130,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -486,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -717,6 +737,92 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>03-03-2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>03:49</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>69176.2</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>69200</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>71200</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>66800</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>177.5</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>277.5</v>
+      </c>
+      <c r="Q3" s="8" t="n">
+        <v>-166</v>
+      </c>
+      <c r="R3" s="9" t="n">
+        <v>-15178</v>
+      </c>
+      <c r="S3" s="10" t="n">
+        <v>-150</v>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>SL — Combined 2.5x (intraday @ 15:01)</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>11h 12m</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>DRY RUN</t>
+        </is>
+      </c>
+      <c r="W3" s="7">
+        <f>W2+R3</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[EXIT] 2026-03-04 11:57 UTC
</commit_message>
<xml_diff>
--- a/trade_tracker.xlsx
+++ b/trade_tracker.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -823,6 +823,92 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>04-03-2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>03:49</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>68257</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>68200</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>71200</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>65200</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="Q4" s="8" t="n">
+        <v>-75</v>
+      </c>
+      <c r="R4" s="9" t="n">
+        <v>-6872</v>
+      </c>
+      <c r="S4" s="10" t="n">
+        <v>-150</v>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>SL — Combined 2.5x (intraday @ 15:12)</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>11h 23m</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>DRY RUN</t>
+        </is>
+      </c>
+      <c r="W4" s="7">
+        <f>W3+R4</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[EXIT] 2026-03-05 12:00 UTC
</commit_message>
<xml_diff>
--- a/trade_tracker.xlsx
+++ b/trade_tracker.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -909,6 +909,92 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>05-03-2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>03:52</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>73277.2</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>73200</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>75200</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>70800</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="R5" s="5" t="n">
+        <v>11514</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>Time Exit — Options Expired OTM (full premium kept)</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>13h 38m</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>DRY RUN</t>
+        </is>
+      </c>
+      <c r="W5" s="7">
+        <f>W4+R5</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[EXIT] 2026-03-07 11:51 UTC
</commit_message>
<xml_diff>
--- a/trade_tracker.xlsx
+++ b/trade_tracker.xlsx
@@ -53,7 +53,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +68,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAEEF3"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +120,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -482,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -704,6 +718,89 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>07-03-2026</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>03:49</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>68321.3</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>68400</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>70400</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>66400</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="R3" s="5" t="n">
+        <v>3213</v>
+      </c>
+      <c r="S3" s="9">
+        <f>S2+R3</f>
+        <v/>
+      </c>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>Early Exit — Premium decayed</t>
+        </is>
+      </c>
+      <c r="U3" s="7" t="inlineStr">
+        <is>
+          <t>13h 32m</t>
+        </is>
+      </c>
+      <c r="V3" s="7" t="inlineStr">
+        <is>
+          <t>DRY RUN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>